<commit_message>
modified csv for input data
filtered on needed chemicals, calculated mean long, lat and alt, summed capacities by chemical
</commit_message>
<xml_diff>
--- a/plants_data/SFI_ALD_Petrochemicals_Sample_EU_NA_Apr_2022.xlsx
+++ b/plants_data/SFI_ALD_Petrochemicals_Sample_EU_NA_Apr_2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\plants_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9976C187-9B33-4E00-BBB3-543BD2517113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AE3B68-1B9D-482F-A9CB-873F60256474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{49FED9BB-E9B4-4298-B606-A2033C4439F2}"/>
   </bookViews>
@@ -31085,16 +31085,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c95907cf-e9f9-4b92-a10f-5d23f887974d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E03E5363D60F6E41BBDBD2986891499D" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="723753e909a658b81c41a8b79ae01792">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c95907cf-e9f9-4b92-a10f-5d23f887974d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e3777ca4d9a00e3a0fcbf4dc5e7e1334" ns2:_="">
     <xsd:import namespace="c95907cf-e9f9-4b92-a10f-5d23f887974d"/>
@@ -31278,6 +31268,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c95907cf-e9f9-4b92-a10f-5d23f887974d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -31288,6 +31288,24 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82F1485-9B46-4DE7-8EF4-68C318268E4B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c95907cf-e9f9-4b92-a10f-5d23f887974d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55D8B328-D93F-4E0D-94E2-653BFEE7AE74}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -31306,24 +31324,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82F1485-9B46-4DE7-8EF4-68C318268E4B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c95907cf-e9f9-4b92-a10f-5d23f887974d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DF01CBF-A5C4-4282-859D-8EAB800F0387}">
   <ds:schemaRefs>

</xml_diff>